<commit_message>
auto update (Home Full Ver)
</commit_message>
<xml_diff>
--- a/weekly_performance.xlsx
+++ b/weekly_performance.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S178"/>
+  <dimension ref="A1:S179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6543,128 +6543,122 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="inlineStr">
+      <c r="A148" t="inlineStr">
         <is>
           <t>통합ETF</t>
         </is>
       </c>
-      <c r="B148" s="2" t="inlineStr">
+      <c r="B148" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C148" s="2" t="inlineStr">
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>09/21~09/25</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" t="n">
+        <v>100</v>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="n">
+        <v>28</v>
+      </c>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="n">
+        <v>2.425</v>
+      </c>
+      <c r="N148" t="n">
+        <v>37246</v>
+      </c>
+      <c r="O148" t="inlineStr"/>
+      <c r="P148" t="n">
+        <v>-106352</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>4918</v>
+      </c>
+      <c r="R148" t="n">
+        <v>-101433</v>
+      </c>
+      <c r="S148" t="n">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>통합ETF</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D148" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="E148" s="2" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="F148" s="2" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="G148" s="2" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="H148" s="2" t="n">
+      <c r="D149" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E149" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F149" s="2" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="G149" s="2" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="H149" s="2" t="n">
         <v>1.49</v>
       </c>
-      <c r="I148" s="2" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="J148" s="2" t="n">
+      <c r="I149" s="2" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="J149" s="2" t="n">
         <v>4.05</v>
       </c>
-      <c r="K148" s="2" t="n">
-        <v>10.75</v>
-      </c>
-      <c r="L148" s="2" t="n">
+      <c r="K149" s="2" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="L149" s="2" t="n">
         <v>7.47</v>
       </c>
-      <c r="M148" s="2" t="n">
-        <v>-0.9419999999999999</v>
-      </c>
-      <c r="N148" s="2" t="n">
-        <v>-26899</v>
-      </c>
-      <c r="O148" s="2" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="P148" s="2" t="n">
-        <v>-504757</v>
-      </c>
-      <c r="Q148" s="2" t="n">
-        <v>40759</v>
-      </c>
-      <c r="R148" s="2" t="n">
-        <v>-463999</v>
-      </c>
-      <c r="S148" s="2" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>수동합계</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>혼합</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>07/27~07/31</t>
-        </is>
-      </c>
-      <c r="D150" t="n">
-        <v>9</v>
-      </c>
-      <c r="E150" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="F150" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="G150" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="H150" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="I150" t="n">
-        <v>3.38</v>
-      </c>
-      <c r="J150" t="n">
-        <v>7.04</v>
-      </c>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
-      <c r="M150" t="n">
-        <v>-1.213</v>
-      </c>
-      <c r="N150" t="n">
-        <v>-744</v>
-      </c>
-      <c r="O150" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="P150" t="n">
-        <v>-6692</v>
-      </c>
-      <c r="Q150" t="n">
-        <v>2139</v>
-      </c>
-      <c r="R150" t="n">
-        <v>-4553</v>
-      </c>
-      <c r="S150" t="n">
-        <v>1415</v>
-      </c>
+      <c r="M149" s="2" t="n">
+        <v>-0.774</v>
+      </c>
+      <c r="N149" s="2" t="n">
+        <v>-23692</v>
+      </c>
+      <c r="O149" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="P149" s="2" t="n">
+        <v>-611109</v>
+      </c>
+      <c r="Q149" s="2" t="n">
+        <v>45677</v>
+      </c>
+      <c r="R149" s="2" t="n">
+        <v>-565432</v>
+      </c>
+      <c r="S149" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6679,44 +6673,52 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>08/10~08/14</t>
+          <t>07/27~07/31</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E151" t="n">
-        <v>100</v>
-      </c>
-      <c r="F151" t="inlineStr"/>
+        <v>55.6</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0.6899999999999999</v>
+      </c>
       <c r="G151" t="n">
-        <v>8.56</v>
-      </c>
-      <c r="H151" t="inlineStr"/>
+        <v>1.17</v>
+      </c>
+      <c r="H151" t="n">
+        <v>4.19</v>
+      </c>
       <c r="I151" t="n">
-        <v>12.69</v>
-      </c>
-      <c r="J151" t="inlineStr"/>
+        <v>3.38</v>
+      </c>
+      <c r="J151" t="n">
+        <v>7.04</v>
+      </c>
       <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="n">
-        <v>8.56</v>
+        <v>-1.213</v>
       </c>
       <c r="N151" t="n">
-        <v>57466</v>
-      </c>
-      <c r="O151" t="inlineStr"/>
+        <v>-744</v>
+      </c>
+      <c r="O151" t="n">
+        <v>0.86</v>
+      </c>
       <c r="P151" t="n">
-        <v>114933</v>
+        <v>-6692</v>
       </c>
       <c r="Q151" t="n">
-        <v>667</v>
+        <v>2139</v>
       </c>
       <c r="R151" t="n">
-        <v>115600</v>
+        <v>-4553</v>
       </c>
       <c r="S151" t="n">
-        <v>1411</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="152">
@@ -6732,44 +6734,44 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>08/24~08/28</t>
+          <t>08/10~08/14</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E152" t="n">
         <v>100</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="n">
-        <v>4.03</v>
+        <v>8.56</v>
       </c>
       <c r="H152" t="inlineStr"/>
       <c r="I152" t="n">
-        <v>4.03</v>
+        <v>12.69</v>
       </c>
       <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="n">
-        <v>4.029</v>
+        <v>8.56</v>
       </c>
       <c r="N152" t="n">
-        <v>35381</v>
+        <v>57466</v>
       </c>
       <c r="O152" t="inlineStr"/>
       <c r="P152" t="n">
-        <v>35381</v>
+        <v>114933</v>
       </c>
       <c r="Q152" t="n">
-        <v>269</v>
+        <v>667</v>
       </c>
       <c r="R152" t="n">
-        <v>35650</v>
+        <v>115600</v>
       </c>
       <c r="S152" t="n">
-        <v>1383</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="153">
@@ -6785,173 +6787,161 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>08/31~09/04</t>
+          <t>08/24~08/28</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E153" t="n">
-        <v>0</v>
-      </c>
-      <c r="F153" t="n">
-        <v>0</v>
-      </c>
-      <c r="G153" t="inlineStr"/>
-      <c r="H153" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="n">
-        <v>2.96</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="n">
+        <v>4.029</v>
+      </c>
+      <c r="N153" t="n">
+        <v>35381</v>
+      </c>
+      <c r="O153" t="inlineStr"/>
+      <c r="P153" t="n">
+        <v>35381</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>269</v>
+      </c>
+      <c r="R153" t="n">
+        <v>35650</v>
+      </c>
+      <c r="S153" t="n">
+        <v>1383</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>수동합계</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>혼합</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>08/31~09/04</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>2</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="n">
         <v>-2.191</v>
       </c>
-      <c r="N153" t="n">
+      <c r="N154" t="n">
         <v>-21127</v>
       </c>
-      <c r="O153" t="n">
-        <v>0</v>
-      </c>
-      <c r="P153" t="n">
+      <c r="O154" t="n">
+        <v>0</v>
+      </c>
+      <c r="P154" t="n">
         <v>-59156</v>
       </c>
-      <c r="Q153" t="n">
+      <c r="Q154" t="n">
         <v>756</v>
       </c>
-      <c r="R153" t="n">
+      <c r="R154" t="n">
         <v>-58400</v>
       </c>
-      <c r="S153" t="n">
+      <c r="S154" t="n">
         <v>1369</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="2" t="inlineStr">
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
         <is>
           <t>수동합계</t>
         </is>
       </c>
-      <c r="B154" s="2" t="inlineStr">
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>혼합</t>
         </is>
       </c>
-      <c r="C154" s="2" t="inlineStr">
+      <c r="C155" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D154" s="2" t="n">
+      <c r="D155" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E154" s="2" t="n">
+      <c r="E155" s="2" t="n">
         <v>57.1</v>
       </c>
-      <c r="F154" s="2" t="n">
+      <c r="F155" s="2" t="n">
         <v>1.59</v>
       </c>
-      <c r="G154" s="2" t="n">
+      <c r="G155" s="2" t="n">
         <v>3.38</v>
       </c>
-      <c r="H154" s="2" t="n">
+      <c r="H155" s="2" t="n">
         <v>3.53</v>
       </c>
-      <c r="I154" s="2" t="n">
+      <c r="I155" s="2" t="n">
         <v>12.69</v>
       </c>
-      <c r="J154" s="2" t="n">
+      <c r="J155" s="2" t="n">
         <v>7.04</v>
       </c>
-      <c r="K154" s="2" t="inlineStr"/>
-      <c r="L154" s="2" t="inlineStr"/>
-      <c r="M154" s="2" t="n">
+      <c r="K155" s="2" t="inlineStr"/>
+      <c r="L155" s="2" t="inlineStr"/>
+      <c r="M155" s="2" t="n">
         <v>0.418</v>
       </c>
-      <c r="N154" s="2" t="n">
+      <c r="N155" s="2" t="n">
         <v>7241</v>
       </c>
-      <c r="O154" s="2" t="n">
+      <c r="O155" s="2" t="n">
         <v>2.12</v>
       </c>
-      <c r="P154" s="2" t="n">
+      <c r="P155" s="2" t="n">
         <v>84466</v>
       </c>
-      <c r="Q154" s="2" t="n">
+      <c r="Q155" s="2" t="n">
         <v>3831</v>
       </c>
-      <c r="R154" s="2" t="n">
+      <c r="R155" s="2" t="n">
         <v>88297</v>
       </c>
-      <c r="S154" s="2" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>수동매매</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>07/27~07/31</t>
-        </is>
-      </c>
-      <c r="D156" t="n">
-        <v>9</v>
-      </c>
-      <c r="E156" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="F156" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="G156" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="H156" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="I156" t="n">
-        <v>3.38</v>
-      </c>
-      <c r="J156" t="n">
-        <v>7.04</v>
-      </c>
-      <c r="K156" t="n">
-        <v>3</v>
-      </c>
-      <c r="L156" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="M156" t="n">
-        <v>-1.213</v>
-      </c>
-      <c r="N156" t="n">
-        <v>-744</v>
-      </c>
-      <c r="O156" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="P156" t="n">
-        <v>-6692</v>
-      </c>
-      <c r="Q156" t="n">
-        <v>2139</v>
-      </c>
-      <c r="R156" t="n">
-        <v>-4553</v>
-      </c>
-      <c r="S156" t="n">
-        <v>1415</v>
-      </c>
+      <c r="S155" s="2" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6966,46 +6956,56 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>08/10~08/14</t>
+          <t>07/27~07/31</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E157" t="n">
-        <v>100</v>
-      </c>
-      <c r="F157" t="inlineStr"/>
+        <v>55.6</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0.6899999999999999</v>
+      </c>
       <c r="G157" t="n">
-        <v>8.56</v>
-      </c>
-      <c r="H157" t="inlineStr"/>
+        <v>1.17</v>
+      </c>
+      <c r="H157" t="n">
+        <v>4.19</v>
+      </c>
       <c r="I157" t="n">
-        <v>12.69</v>
-      </c>
-      <c r="J157" t="inlineStr"/>
+        <v>3.38</v>
+      </c>
+      <c r="J157" t="n">
+        <v>7.04</v>
+      </c>
       <c r="K157" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L157" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="L157" t="n">
+        <v>1.75</v>
+      </c>
       <c r="M157" t="n">
-        <v>8.56</v>
+        <v>-1.213</v>
       </c>
       <c r="N157" t="n">
-        <v>57466</v>
-      </c>
-      <c r="O157" t="inlineStr"/>
+        <v>-744</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0.86</v>
+      </c>
       <c r="P157" t="n">
-        <v>114933</v>
+        <v>-6692</v>
       </c>
       <c r="Q157" t="n">
-        <v>667</v>
+        <v>2139</v>
       </c>
       <c r="R157" t="n">
-        <v>115600</v>
+        <v>-4553</v>
       </c>
       <c r="S157" t="n">
-        <v>1411</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="158">
@@ -7021,46 +7021,46 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>08/24~08/28</t>
+          <t>08/10~08/14</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E158" t="n">
         <v>100</v>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="n">
-        <v>4.03</v>
+        <v>8.56</v>
       </c>
       <c r="H158" t="inlineStr"/>
       <c r="I158" t="n">
-        <v>4.03</v>
+        <v>12.69</v>
       </c>
       <c r="J158" t="inlineStr"/>
       <c r="K158" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="n">
-        <v>4.029</v>
+        <v>8.56</v>
       </c>
       <c r="N158" t="n">
-        <v>35381</v>
+        <v>57466</v>
       </c>
       <c r="O158" t="inlineStr"/>
       <c r="P158" t="n">
-        <v>35381</v>
+        <v>114933</v>
       </c>
       <c r="Q158" t="n">
-        <v>269</v>
+        <v>667</v>
       </c>
       <c r="R158" t="n">
-        <v>35650</v>
+        <v>115600</v>
       </c>
       <c r="S158" t="n">
-        <v>1383</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="159">
@@ -7076,239 +7076,251 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
+          <t>08/24~08/28</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>1</v>
+      </c>
+      <c r="E159" t="n">
+        <v>100</v>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="n">
+        <v>1</v>
+      </c>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="n">
+        <v>4.029</v>
+      </c>
+      <c r="N159" t="n">
+        <v>35381</v>
+      </c>
+      <c r="O159" t="inlineStr"/>
+      <c r="P159" t="n">
+        <v>35381</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>269</v>
+      </c>
+      <c r="R159" t="n">
+        <v>35650</v>
+      </c>
+      <c r="S159" t="n">
+        <v>1383</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>수동매매</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
           <t>08/31~09/04</t>
         </is>
       </c>
-      <c r="D159" t="n">
+      <c r="D160" t="n">
         <v>2</v>
       </c>
-      <c r="E159" t="n">
-        <v>0</v>
-      </c>
-      <c r="F159" t="n">
-        <v>0</v>
-      </c>
-      <c r="G159" t="inlineStr"/>
-      <c r="H159" t="n">
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="n">
         <v>2.19</v>
       </c>
-      <c r="I159" t="inlineStr"/>
-      <c r="J159" t="n">
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="n">
         <v>2.96</v>
       </c>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="n">
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="n">
         <v>6.5</v>
       </c>
-      <c r="M159" t="n">
+      <c r="M160" t="n">
         <v>-2.191</v>
       </c>
-      <c r="N159" t="n">
+      <c r="N160" t="n">
         <v>-21127</v>
       </c>
-      <c r="O159" t="n">
-        <v>0</v>
-      </c>
-      <c r="P159" t="n">
+      <c r="O160" t="n">
+        <v>0</v>
+      </c>
+      <c r="P160" t="n">
         <v>-59156</v>
       </c>
-      <c r="Q159" t="n">
+      <c r="Q160" t="n">
         <v>756</v>
       </c>
-      <c r="R159" t="n">
+      <c r="R160" t="n">
         <v>-58400</v>
       </c>
-      <c r="S159" t="n">
+      <c r="S160" t="n">
         <v>1369</v>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" s="2" t="inlineStr">
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
         <is>
           <t>수동매매</t>
         </is>
       </c>
-      <c r="B160" s="2" t="inlineStr">
+      <c r="B161" s="2" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C160" s="2" t="inlineStr">
+      <c r="C161" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D160" s="2" t="n">
+      <c r="D161" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E160" s="2" t="n">
+      <c r="E161" s="2" t="n">
         <v>57.1</v>
       </c>
-      <c r="F160" s="2" t="n">
+      <c r="F161" s="2" t="n">
         <v>1.59</v>
       </c>
-      <c r="G160" s="2" t="n">
+      <c r="G161" s="2" t="n">
         <v>3.38</v>
       </c>
-      <c r="H160" s="2" t="n">
+      <c r="H161" s="2" t="n">
         <v>3.53</v>
       </c>
-      <c r="I160" s="2" t="n">
+      <c r="I161" s="2" t="n">
         <v>12.69</v>
       </c>
-      <c r="J160" s="2" t="n">
+      <c r="J161" s="2" t="n">
         <v>7.04</v>
       </c>
-      <c r="K160" s="2" t="n">
+      <c r="K161" s="2" t="n">
         <v>3.12</v>
       </c>
-      <c r="L160" s="2" t="n">
+      <c r="L161" s="2" t="n">
         <v>3.33</v>
       </c>
-      <c r="M160" s="2" t="n">
+      <c r="M161" s="2" t="n">
         <v>0.418</v>
       </c>
-      <c r="N160" s="2" t="n">
+      <c r="N161" s="2" t="n">
         <v>7241</v>
       </c>
-      <c r="O160" s="2" t="n">
+      <c r="O161" s="2" t="n">
         <v>2.12</v>
       </c>
-      <c r="P160" s="2" t="n">
+      <c r="P161" s="2" t="n">
         <v>84466</v>
       </c>
-      <c r="Q160" s="2" t="n">
+      <c r="Q161" s="2" t="n">
         <v>3831</v>
       </c>
-      <c r="R160" s="2" t="n">
+      <c r="R161" s="2" t="n">
         <v>88297</v>
       </c>
-      <c r="S160" s="2" t="inlineStr"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="2" t="inlineStr">
+      <c r="S161" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
         <is>
           <t>미국수동</t>
         </is>
       </c>
-      <c r="B162" s="2" t="inlineStr">
+      <c r="B163" s="2" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr">
+      <c r="C163" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D162" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E162" s="2" t="inlineStr"/>
-      <c r="F162" s="2" t="inlineStr"/>
-      <c r="G162" s="2" t="inlineStr"/>
-      <c r="H162" s="2" t="inlineStr"/>
-      <c r="I162" s="2" t="inlineStr"/>
-      <c r="J162" s="2" t="inlineStr"/>
-      <c r="K162" s="2" t="inlineStr"/>
-      <c r="L162" s="2" t="inlineStr"/>
-      <c r="M162" s="2" t="inlineStr"/>
-      <c r="N162" s="2" t="inlineStr"/>
-      <c r="O162" s="2" t="inlineStr"/>
-      <c r="P162" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q162" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R162" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S162" s="2" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="2" t="inlineStr">
+      <c r="D163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E163" s="2" t="inlineStr"/>
+      <c r="F163" s="2" t="inlineStr"/>
+      <c r="G163" s="2" t="inlineStr"/>
+      <c r="H163" s="2" t="inlineStr"/>
+      <c r="I163" s="2" t="inlineStr"/>
+      <c r="J163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr"/>
+      <c r="L163" s="2" t="inlineStr"/>
+      <c r="M163" s="2" t="inlineStr"/>
+      <c r="N163" s="2" t="inlineStr"/>
+      <c r="O163" s="2" t="inlineStr"/>
+      <c r="P163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S163" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
         <is>
           <t>기타(8042)</t>
         </is>
       </c>
-      <c r="B164" s="2" t="inlineStr">
+      <c r="B165" s="2" t="inlineStr">
         <is>
           <t>분</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D164" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E164" s="2" t="inlineStr"/>
-      <c r="F164" s="2" t="inlineStr"/>
-      <c r="G164" s="2" t="inlineStr"/>
-      <c r="H164" s="2" t="inlineStr"/>
-      <c r="I164" s="2" t="inlineStr"/>
-      <c r="J164" s="2" t="inlineStr"/>
-      <c r="K164" s="2" t="inlineStr"/>
-      <c r="L164" s="2" t="inlineStr"/>
-      <c r="M164" s="2" t="inlineStr"/>
-      <c r="N164" s="2" t="inlineStr"/>
-      <c r="O164" s="2" t="inlineStr"/>
-      <c r="P164" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q164" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R164" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S164" s="2" t="inlineStr"/>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>2X단타_시딩</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>08/17~08/21</t>
-        </is>
-      </c>
-      <c r="D166" t="n">
-        <v>0</v>
-      </c>
-      <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
-      <c r="I166" t="inlineStr"/>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
-      <c r="M166" t="inlineStr"/>
-      <c r="N166" t="inlineStr"/>
-      <c r="O166" t="inlineStr"/>
-      <c r="P166" t="n">
-        <v>51315</v>
-      </c>
-      <c r="Q166" t="n">
-        <v>1370</v>
-      </c>
-      <c r="R166" t="n">
-        <v>52685</v>
-      </c>
-      <c r="S166" t="n">
-        <v>1373</v>
-      </c>
+      <c r="D165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E165" s="2" t="inlineStr"/>
+      <c r="F165" s="2" t="inlineStr"/>
+      <c r="G165" s="2" t="inlineStr"/>
+      <c r="H165" s="2" t="inlineStr"/>
+      <c r="I165" s="2" t="inlineStr"/>
+      <c r="J165" s="2" t="inlineStr"/>
+      <c r="K165" s="2" t="inlineStr"/>
+      <c r="L165" s="2" t="inlineStr"/>
+      <c r="M165" s="2" t="inlineStr"/>
+      <c r="N165" s="2" t="inlineStr"/>
+      <c r="O165" s="2" t="inlineStr"/>
+      <c r="P165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S165" s="2" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7323,7 +7335,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>08/31~09/04</t>
+          <t>08/17~08/21</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -7341,16 +7353,16 @@
       <c r="N167" t="inlineStr"/>
       <c r="O167" t="inlineStr"/>
       <c r="P167" t="n">
-        <v>-69677</v>
+        <v>51315</v>
       </c>
       <c r="Q167" t="n">
-        <v>262</v>
+        <v>1370</v>
       </c>
       <c r="R167" t="n">
-        <v>-69415</v>
+        <v>52685</v>
       </c>
       <c r="S167" t="n">
-        <v>1369</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="168">
@@ -7366,456 +7378,499 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
+          <t>08/31~09/04</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>0</v>
+      </c>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr"/>
+      <c r="M168" t="inlineStr"/>
+      <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr"/>
+      <c r="P168" t="n">
+        <v>-69677</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>262</v>
+      </c>
+      <c r="R168" t="n">
+        <v>-69415</v>
+      </c>
+      <c r="S168" t="n">
+        <v>1369</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2X단타_시딩</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
           <t>09/07~09/11</t>
         </is>
       </c>
-      <c r="D168" t="n">
+      <c r="D169" t="n">
         <v>1</v>
       </c>
-      <c r="E168" t="n">
-        <v>0</v>
-      </c>
-      <c r="F168" t="n">
-        <v>0</v>
-      </c>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="n">
+      <c r="E169" t="n">
+        <v>0</v>
+      </c>
+      <c r="F169" t="n">
+        <v>0</v>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="n">
         <v>0.61</v>
       </c>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="n">
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="n">
         <v>0.61</v>
       </c>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="n">
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="n">
         <v>21</v>
       </c>
-      <c r="M168" t="n">
+      <c r="M169" t="n">
         <v>-0.612</v>
       </c>
-      <c r="N168" t="n">
+      <c r="N169" t="n">
         <v>-37549</v>
       </c>
-      <c r="O168" t="n">
-        <v>0</v>
-      </c>
-      <c r="P168" t="n">
+      <c r="O169" t="n">
+        <v>0</v>
+      </c>
+      <c r="P169" t="n">
         <v>-19186</v>
       </c>
-      <c r="Q168" t="n">
+      <c r="Q169" t="n">
         <v>201</v>
       </c>
-      <c r="R168" t="n">
+      <c r="R169" t="n">
         <v>-18985</v>
       </c>
-      <c r="S168" t="n">
+      <c r="S169" t="n">
         <v>1338</v>
       </c>
     </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
         <is>
           <t>2X단타_시딩</t>
         </is>
       </c>
-      <c r="B169" s="2" t="inlineStr">
+      <c r="B170" s="2" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C169" s="2" t="inlineStr">
+      <c r="C170" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D169" s="2" t="n">
+      <c r="D170" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E169" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F169" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G169" s="2" t="inlineStr"/>
-      <c r="H169" s="2" t="n">
+      <c r="E170" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" s="2" t="inlineStr"/>
+      <c r="H170" s="2" t="n">
         <v>0.61</v>
       </c>
-      <c r="I169" s="2" t="inlineStr"/>
-      <c r="J169" s="2" t="n">
+      <c r="I170" s="2" t="inlineStr"/>
+      <c r="J170" s="2" t="n">
         <v>0.61</v>
       </c>
-      <c r="K169" s="2" t="inlineStr"/>
-      <c r="L169" s="2" t="n">
+      <c r="K170" s="2" t="inlineStr"/>
+      <c r="L170" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="M169" s="2" t="n">
+      <c r="M170" s="2" t="n">
         <v>-0.612</v>
       </c>
-      <c r="N169" s="2" t="n">
+      <c r="N170" s="2" t="n">
         <v>-37549</v>
       </c>
-      <c r="O169" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P169" s="2" t="n">
+      <c r="O170" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P170" s="2" t="n">
         <v>-37548</v>
       </c>
-      <c r="Q169" s="2" t="n">
+      <c r="Q170" s="2" t="n">
         <v>1833</v>
       </c>
-      <c r="R169" s="2" t="n">
+      <c r="R170" s="2" t="n">
         <v>-35715</v>
       </c>
-      <c r="S169" s="2" t="inlineStr"/>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
+      <c r="S170" s="2" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
         <is>
           <t>수동매매_시딩</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr">
+      <c r="B172" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
+      <c r="C172" t="inlineStr">
         <is>
           <t>08/17~08/21</t>
         </is>
       </c>
-      <c r="D171" t="n">
+      <c r="D172" t="n">
         <v>1</v>
       </c>
-      <c r="E171" t="n">
-        <v>0</v>
-      </c>
-      <c r="F171" t="n">
-        <v>0</v>
-      </c>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="n">
+      <c r="E172" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="I171" t="inlineStr"/>
-      <c r="J171" t="n">
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="n">
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="n">
         <v>3</v>
       </c>
-      <c r="M171" t="n">
+      <c r="M172" t="n">
         <v>-8.304</v>
       </c>
-      <c r="N171" t="n">
+      <c r="N172" t="n">
         <v>-74087</v>
       </c>
-      <c r="O171" t="n">
-        <v>0</v>
-      </c>
-      <c r="P171" t="n">
+      <c r="O172" t="n">
+        <v>0</v>
+      </c>
+      <c r="P172" t="n">
         <v>-74087</v>
       </c>
-      <c r="Q171" t="n">
+      <c r="Q172" t="n">
         <v>257</v>
       </c>
-      <c r="R171" t="n">
+      <c r="R172" t="n">
         <v>-73830</v>
       </c>
-      <c r="S171" t="n">
+      <c r="S172" t="n">
         <v>1373</v>
       </c>
     </row>
-    <row r="172">
-      <c r="A172" s="2" t="inlineStr">
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
         <is>
           <t>수동매매_시딩</t>
         </is>
       </c>
-      <c r="B172" s="2" t="inlineStr">
+      <c r="B173" s="2" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C172" s="2" t="inlineStr">
+      <c r="C173" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D172" s="2" t="n">
+      <c r="D173" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E172" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F172" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G172" s="2" t="inlineStr"/>
-      <c r="H172" s="2" t="n">
+      <c r="E173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G173" s="2" t="inlineStr"/>
+      <c r="H173" s="2" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="I172" s="2" t="inlineStr"/>
-      <c r="J172" s="2" t="n">
+      <c r="I173" s="2" t="inlineStr"/>
+      <c r="J173" s="2" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="K172" s="2" t="inlineStr"/>
-      <c r="L172" s="2" t="n">
+      <c r="K173" s="2" t="inlineStr"/>
+      <c r="L173" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M172" s="2" t="n">
+      <c r="M173" s="2" t="n">
         <v>-8.304</v>
       </c>
-      <c r="N172" s="2" t="n">
+      <c r="N173" s="2" t="n">
         <v>-74087</v>
       </c>
-      <c r="O172" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P172" s="2" t="n">
+      <c r="O173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P173" s="2" t="n">
         <v>-74087</v>
       </c>
-      <c r="Q172" s="2" t="n">
+      <c r="Q173" s="2" t="n">
         <v>257</v>
       </c>
-      <c r="R172" s="2" t="n">
+      <c r="R173" s="2" t="n">
         <v>-73830</v>
       </c>
-      <c r="S172" s="2" t="inlineStr"/>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
+      <c r="S173" s="2" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
         <is>
           <t>주도주_시딩</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B175" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C175" t="inlineStr">
         <is>
           <t>08/17~08/21</t>
         </is>
       </c>
-      <c r="D174" t="n">
+      <c r="D175" t="n">
         <v>1</v>
       </c>
-      <c r="E174" t="n">
-        <v>0</v>
-      </c>
-      <c r="F174" t="n">
-        <v>0</v>
-      </c>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="n">
+      <c r="E175" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" t="n">
+        <v>0</v>
+      </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="n">
         <v>4.6</v>
       </c>
-      <c r="I174" t="inlineStr"/>
-      <c r="J174" t="n">
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="n">
         <v>4.6</v>
       </c>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="n">
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="n">
         <v>3</v>
       </c>
-      <c r="M174" t="n">
+      <c r="M175" t="n">
         <v>-4.602</v>
       </c>
-      <c r="N174" t="n">
+      <c r="N175" t="n">
         <v>-29689</v>
       </c>
-      <c r="O174" t="n">
-        <v>0</v>
-      </c>
-      <c r="P174" t="n">
+      <c r="O175" t="n">
+        <v>0</v>
+      </c>
+      <c r="P175" t="n">
         <v>-29689</v>
       </c>
-      <c r="Q174" t="n">
+      <c r="Q175" t="n">
         <v>189</v>
       </c>
-      <c r="R174" t="n">
+      <c r="R175" t="n">
         <v>-29500</v>
       </c>
-      <c r="S174" t="n">
+      <c r="S175" t="n">
         <v>1373</v>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="2" t="inlineStr">
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
         <is>
           <t>주도주_시딩</t>
         </is>
       </c>
-      <c r="B175" s="2" t="inlineStr">
+      <c r="B176" s="2" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr">
+      <c r="C176" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D175" s="2" t="n">
+      <c r="D176" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E175" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F175" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G175" s="2" t="inlineStr"/>
-      <c r="H175" s="2" t="n">
+      <c r="E176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" s="2" t="inlineStr"/>
+      <c r="H176" s="2" t="n">
         <v>4.6</v>
       </c>
-      <c r="I175" s="2" t="inlineStr"/>
-      <c r="J175" s="2" t="n">
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="n">
         <v>4.6</v>
       </c>
-      <c r="K175" s="2" t="inlineStr"/>
-      <c r="L175" s="2" t="n">
+      <c r="K176" s="2" t="inlineStr"/>
+      <c r="L176" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M175" s="2" t="n">
+      <c r="M176" s="2" t="n">
         <v>-4.602</v>
       </c>
-      <c r="N175" s="2" t="n">
+      <c r="N176" s="2" t="n">
         <v>-29689</v>
       </c>
-      <c r="O175" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P175" s="2" t="n">
+      <c r="O176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P176" s="2" t="n">
         <v>-29689</v>
       </c>
-      <c r="Q175" s="2" t="n">
+      <c r="Q176" s="2" t="n">
         <v>189</v>
       </c>
-      <c r="R175" s="2" t="n">
+      <c r="R176" s="2" t="n">
         <v>-29500</v>
       </c>
-      <c r="S175" s="2" t="inlineStr"/>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
+      <c r="S176" s="2" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
         <is>
           <t>통합ETF_시딩</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B178" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C178" t="inlineStr">
         <is>
           <t>08/17~08/21</t>
         </is>
       </c>
-      <c r="D177" t="n">
+      <c r="D178" t="n">
         <v>1</v>
       </c>
-      <c r="E177" t="n">
-        <v>0</v>
-      </c>
-      <c r="F177" t="n">
-        <v>0</v>
-      </c>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="n">
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" t="n">
+        <v>0</v>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="n">
         <v>0.87</v>
       </c>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="n">
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="n">
         <v>0.87</v>
       </c>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="n">
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="n">
         <v>3</v>
       </c>
-      <c r="M177" t="n">
+      <c r="M178" t="n">
         <v>-0.867</v>
       </c>
-      <c r="N177" t="n">
+      <c r="N178" t="n">
         <v>-29188</v>
       </c>
-      <c r="O177" t="n">
-        <v>0</v>
-      </c>
-      <c r="P177" t="n">
+      <c r="O178" t="n">
+        <v>0</v>
+      </c>
+      <c r="P178" t="n">
         <v>-29188</v>
       </c>
-      <c r="Q177" t="n">
+      <c r="Q178" t="n">
         <v>2950</v>
       </c>
-      <c r="R177" t="n">
+      <c r="R178" t="n">
         <v>-26238</v>
       </c>
-      <c r="S177" t="n">
+      <c r="S178" t="n">
         <v>1373</v>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>통합ETF_시딩</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="D178" s="2" t="n">
+      <c r="D179" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E178" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F178" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G178" s="2" t="inlineStr"/>
-      <c r="H178" s="2" t="n">
+      <c r="E179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G179" s="2" t="inlineStr"/>
+      <c r="H179" s="2" t="n">
         <v>0.87</v>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
-      <c r="J178" s="2" t="n">
+      <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="n">
         <v>0.87</v>
       </c>
-      <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="2" t="n">
+      <c r="K179" s="2" t="inlineStr"/>
+      <c r="L179" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M178" s="2" t="n">
+      <c r="M179" s="2" t="n">
         <v>-0.867</v>
       </c>
-      <c r="N178" s="2" t="n">
+      <c r="N179" s="2" t="n">
         <v>-29188</v>
       </c>
-      <c r="O178" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P178" s="2" t="n">
+      <c r="O179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P179" s="2" t="n">
         <v>-29188</v>
       </c>
-      <c r="Q178" s="2" t="n">
+      <c r="Q179" s="2" t="n">
         <v>2950</v>
       </c>
-      <c r="R178" s="2" t="n">
+      <c r="R179" s="2" t="n">
         <v>-26238</v>
       </c>
-      <c r="S178" s="2" t="inlineStr"/>
+      <c r="S179" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto update (Company KR Ver)
</commit_message>
<xml_diff>
--- a/weekly_performance.xlsx
+++ b/weekly_performance.xlsx
@@ -1568,16 +1568,16 @@
         <v>0.91</v>
       </c>
       <c r="P18" t="n">
-        <v>14255</v>
+        <v>14239</v>
       </c>
       <c r="Q18" t="n">
         <v>1300</v>
       </c>
       <c r="R18" t="n">
-        <v>15555</v>
+        <v>15539</v>
       </c>
       <c r="S18" t="n">
-        <v>1360</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="19">
@@ -1629,13 +1629,13 @@
         <v>0.9</v>
       </c>
       <c r="P19" s="2" t="n">
-        <v>-179349</v>
+        <v>-179365</v>
       </c>
       <c r="Q19" s="2" t="n">
         <v>93880</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>-85468</v>
+        <v>-85484</v>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
     </row>
@@ -4148,7 +4148,7 @@
         <v>15290</v>
       </c>
       <c r="S77" t="n">
-        <v>1360</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="78">
@@ -4397,7 +4397,7 @@
         <v>-12750</v>
       </c>
       <c r="S85" t="n">
-        <v>1360</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="86">
@@ -6712,7 +6712,7 @@
         <v>6858</v>
       </c>
       <c r="S150" t="n">
-        <v>1360</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="151">
@@ -6895,7 +6895,7 @@
         <v>1285</v>
       </c>
       <c r="S154" t="n">
-        <v>1360</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="155">
@@ -7035,16 +7035,16 @@
       <c r="N158" t="inlineStr"/>
       <c r="O158" t="inlineStr"/>
       <c r="P158" t="n">
-        <v>2748</v>
+        <v>2732</v>
       </c>
       <c r="Q158" t="n">
         <v>21</v>
       </c>
       <c r="R158" t="n">
-        <v>2769</v>
+        <v>2753</v>
       </c>
       <c r="S158" t="n">
-        <v>1360</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="159">
@@ -7078,13 +7078,13 @@
       <c r="N159" s="2" t="inlineStr"/>
       <c r="O159" s="2" t="inlineStr"/>
       <c r="P159" s="2" t="n">
-        <v>3660</v>
+        <v>3644</v>
       </c>
       <c r="Q159" s="2" t="n">
         <v>82</v>
       </c>
       <c r="R159" s="2" t="n">
-        <v>3742</v>
+        <v>3726</v>
       </c>
       <c r="S159" s="2" t="inlineStr"/>
     </row>
@@ -8735,7 +8735,7 @@
         <v>2103</v>
       </c>
       <c r="S197" t="n">
-        <v>1360</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="198">

</xml_diff>